<commit_message>
docs: update Mapping_Field_SLA.xlsx to one-way mapping (doc -> field)
</commit_message>
<xml_diff>
--- a/Mapping_Field_SLA.xlsx
+++ b/Mapping_Field_SLA.xlsx
@@ -405,23 +405,23 @@
     <col min="4" max="4" width="18.83203125" customWidth="1"/>
     <col min="5" max="5" width="58.83203125" customWidth="1"/>
     <col min="6" max="6" width="11.83203125" customWidth="1"/>
-    <col min="7" max="7" width="28.83203125" customWidth="1"/>
+    <col min="7" max="7" width="30.83203125" customWidth="1"/>
     <col min="8" max="8" width="26.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>DANH SÁCH FIELD SLA (tách phẳng) — ĐỒNG BỘ 2 CHIỀU OnlyOffice &lt;-&gt; panel phải form Tạo mới hợp đồng</v>
+        <v>DANH SÁCH FIELD SLA (tách phẳng) — ÁNH XẠ 1 CHIỀU: OnlyOffice (trái) → field (panel phải)</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Nguồn: PL III - Đánh giá chất lượng DV (SLA). "2 chiều" = sửa ở doc cập nhật field &amp; ngược lại. Field nghiệm thu được điền ở panel phải khi nghiệm thu rồi đẩy ngược vào doc.</v>
+        <v>Nguồn: PL III - Đánh giá chất lượng DV (SLA). "✓" = lấy từ tài liệu lúc tạo HĐ; "Nghiệm thu" = điền ở panel phải khi nghiệm thu; "Chọn tay" = nhập trực tiếp.</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Cơ chế neo: mỗi field gắn 1 Content Control (hoặc placeholder {{field_key}}) trong template OnlyOffice. Chống vòng lặp: debounce + so sánh giá trị trước khi ghi (chỉ ghi khi khác).</v>
+        <v>Cơ chế neo: mỗi field gắn 1 Content Control (hoặc placeholder {{field_key}}) trong template OnlyOffice để đọc giá trị đổ sang field.</v>
       </c>
     </row>
     <row r="5">
@@ -444,7 +444,7 @@
         <v>Nguồn Excel</v>
       </c>
       <c r="G5" t="str">
-        <v>Đồng bộ 2 chiều</v>
+        <v>Ánh xạ (1 chiều: doc → field)</v>
       </c>
       <c r="H5" t="str">
         <v>Neo trong tài liệu (anchor)</v>
@@ -470,7 +470,7 @@
         <v>Tên sheet</v>
       </c>
       <c r="G6" t="str">
-        <v>Chọn tay (không sync)</v>
+        <v>Chọn tay</v>
       </c>
       <c r="H6" t="str">
         <v>(không gắn neo)</v>
@@ -496,7 +496,7 @@
         <v>R0c0</v>
       </c>
       <c r="G7" t="str">
-        <v>2 chiều</v>
+        <v>✓</v>
       </c>
       <c r="H7" t="str">
         <v>{{sla_title}}</v>
@@ -522,7 +522,7 @@
         <v>R0c0</v>
       </c>
       <c r="G8" t="str">
-        <v>2 chiều</v>
+        <v>✓</v>
       </c>
       <c r="H8" t="str">
         <v>{{sla_acceptance_no}}</v>
@@ -548,7 +548,7 @@
         <v>R0c0</v>
       </c>
       <c r="G9" t="str">
-        <v>2 chiều</v>
+        <v>✓</v>
       </c>
       <c r="H9" t="str">
         <v>{{sla_acceptance_date}}</v>
@@ -574,7 +574,7 @@
         <v>R2c4</v>
       </c>
       <c r="G10" t="str">
-        <v>2 chiều</v>
+        <v>✓</v>
       </c>
       <c r="H10" t="str">
         <v>{{sla_max_score}}</v>
@@ -600,7 +600,7 @@
         <v>R2c6</v>
       </c>
       <c r="G11" t="str">
-        <v>2 chiều (điền khi nghiệm thu)</v>
+        <v>Nghiệm thu</v>
       </c>
       <c r="H11" t="str">
         <v>{{sla_total_score}}</v>
@@ -626,7 +626,7 @@
         <v>R2c4</v>
       </c>
       <c r="G12" t="str">
-        <v>2 chiều</v>
+        <v>✓</v>
       </c>
       <c r="H12" t="str">
         <v>{{sla_penalty_95_100}}</v>
@@ -652,7 +652,7 @@
         <v>R2c4</v>
       </c>
       <c r="G13" t="str">
-        <v>2 chiều</v>
+        <v>✓</v>
       </c>
       <c r="H13" t="str">
         <v>{{sla_penalty_90_95}}</v>
@@ -678,7 +678,7 @@
         <v>R2c4</v>
       </c>
       <c r="G14" t="str">
-        <v>2 chiều</v>
+        <v>✓</v>
       </c>
       <c r="H14" t="str">
         <v>{{sla_penalty_80_90}}</v>
@@ -704,7 +704,7 @@
         <v>R2c4</v>
       </c>
       <c r="G15" t="str">
-        <v>2 chiều</v>
+        <v>✓</v>
       </c>
       <c r="H15" t="str">
         <v>{{sla_penalty_70_80}}</v>
@@ -730,7 +730,7 @@
         <v>R2c4</v>
       </c>
       <c r="G16" t="str">
-        <v>2 chiều</v>
+        <v>✓</v>
       </c>
       <c r="H16" t="str">
         <v>{{sla_penalty_65_70}}</v>
@@ -756,7 +756,7 @@
         <v>R2c4</v>
       </c>
       <c r="G17" t="str">
-        <v>2 chiều</v>
+        <v>✓</v>
       </c>
       <c r="H17" t="str">
         <v>{{sla_penalty_below_65}}</v>
@@ -782,7 +782,7 @@
         <v>R3c1</v>
       </c>
       <c r="G18" t="str">
-        <v>2 chiều</v>
+        <v>✓</v>
       </c>
       <c r="H18" t="str">
         <v>{{sla_A_name}}</v>
@@ -808,7 +808,7 @@
         <v>R3c4</v>
       </c>
       <c r="G19" t="str">
-        <v>2 chiều</v>
+        <v>✓</v>
       </c>
       <c r="H19" t="str">
         <v>{{sla_A_quota}}</v>
@@ -834,7 +834,7 @@
         <v>R3c5</v>
       </c>
       <c r="G20" t="str">
-        <v>2 chiều</v>
+        <v>✓</v>
       </c>
       <c r="H20" t="str">
         <v>{{sla_A_weight}}</v>
@@ -860,7 +860,7 @@
         <v>R4c1</v>
       </c>
       <c r="G21" t="str">
-        <v>2 chiều</v>
+        <v>✓</v>
       </c>
       <c r="H21" t="str">
         <v>{{sla_A1_name}}</v>
@@ -886,7 +886,7 @@
         <v>R4c2</v>
       </c>
       <c r="G22" t="str">
-        <v>2 chiều</v>
+        <v>✓</v>
       </c>
       <c r="H22" t="str">
         <v>{{sla_A1_requirement}}</v>
@@ -912,7 +912,7 @@
         <v>R4c3</v>
       </c>
       <c r="G23" t="str">
-        <v>2 chiều</v>
+        <v>✓</v>
       </c>
       <c r="H23" t="str">
         <v>{{sla_A1_method}}</v>
@@ -938,7 +938,7 @@
         <v>R4c4</v>
       </c>
       <c r="G24" t="str">
-        <v>2 chiều</v>
+        <v>✓</v>
       </c>
       <c r="H24" t="str">
         <v>{{sla_A1_target}}</v>
@@ -964,7 +964,7 @@
         <v>R4c6</v>
       </c>
       <c r="G25" t="str">
-        <v>2 chiều (điền khi nghiệm thu)</v>
+        <v>Nghiệm thu</v>
       </c>
       <c r="H25" t="str">
         <v>{{sla_A1_score}}</v>
@@ -990,7 +990,7 @@
         <v>R4c7</v>
       </c>
       <c r="G26" t="str">
-        <v>2 chiều (điền khi nghiệm thu)</v>
+        <v>Nghiệm thu</v>
       </c>
       <c r="H26" t="str">
         <v>{{sla_A1_note}}</v>
@@ -1016,7 +1016,7 @@
         <v>R5c1</v>
       </c>
       <c r="G27" t="str">
-        <v>2 chiều</v>
+        <v>✓</v>
       </c>
       <c r="H27" t="str">
         <v>{{sla_B_name}}</v>
@@ -1042,7 +1042,7 @@
         <v>R5c4</v>
       </c>
       <c r="G28" t="str">
-        <v>2 chiều</v>
+        <v>✓</v>
       </c>
       <c r="H28" t="str">
         <v>{{sla_B_quota}}</v>
@@ -1068,7 +1068,7 @@
         <v>R5c5</v>
       </c>
       <c r="G29" t="str">
-        <v>2 chiều</v>
+        <v>✓</v>
       </c>
       <c r="H29" t="str">
         <v>{{sla_B_weight}}</v>
@@ -1094,7 +1094,7 @@
         <v>R6c1</v>
       </c>
       <c r="G30" t="str">
-        <v>2 chiều</v>
+        <v>✓</v>
       </c>
       <c r="H30" t="str">
         <v>{{sla_B1_name}}</v>
@@ -1120,7 +1120,7 @@
         <v>R6c2</v>
       </c>
       <c r="G31" t="str">
-        <v>2 chiều</v>
+        <v>✓</v>
       </c>
       <c r="H31" t="str">
         <v>{{sla_B1_requirement}}</v>
@@ -1146,7 +1146,7 @@
         <v>R6c3</v>
       </c>
       <c r="G32" t="str">
-        <v>2 chiều</v>
+        <v>✓</v>
       </c>
       <c r="H32" t="str">
         <v>{{sla_B1_method}}</v>
@@ -1172,7 +1172,7 @@
         <v>R6c4</v>
       </c>
       <c r="G33" t="str">
-        <v>2 chiều</v>
+        <v>✓</v>
       </c>
       <c r="H33" t="str">
         <v>{{sla_B1_target}}</v>
@@ -1198,7 +1198,7 @@
         <v>R6c6</v>
       </c>
       <c r="G34" t="str">
-        <v>2 chiều (điền khi nghiệm thu)</v>
+        <v>Nghiệm thu</v>
       </c>
       <c r="H34" t="str">
         <v>{{sla_B1_score}}</v>
@@ -1224,7 +1224,7 @@
         <v>R6c7</v>
       </c>
       <c r="G35" t="str">
-        <v>2 chiều (điền khi nghiệm thu)</v>
+        <v>Nghiệm thu</v>
       </c>
       <c r="H35" t="str">
         <v>{{sla_B1_note}}</v>
@@ -1250,7 +1250,7 @@
         <v>R7c1</v>
       </c>
       <c r="G36" t="str">
-        <v>2 chiều</v>
+        <v>✓</v>
       </c>
       <c r="H36" t="str">
         <v>{{sla_C_name}}</v>
@@ -1276,7 +1276,7 @@
         <v>R7c4</v>
       </c>
       <c r="G37" t="str">
-        <v>2 chiều</v>
+        <v>✓</v>
       </c>
       <c r="H37" t="str">
         <v>{{sla_C_quota}}</v>
@@ -1302,7 +1302,7 @@
         <v>R7c5</v>
       </c>
       <c r="G38" t="str">
-        <v>2 chiều</v>
+        <v>✓</v>
       </c>
       <c r="H38" t="str">
         <v>{{sla_C_weight}}</v>
@@ -1328,7 +1328,7 @@
         <v>R8c1</v>
       </c>
       <c r="G39" t="str">
-        <v>2 chiều</v>
+        <v>✓</v>
       </c>
       <c r="H39" t="str">
         <v>{{sla_C1_name}}</v>
@@ -1354,7 +1354,7 @@
         <v>R8c2</v>
       </c>
       <c r="G40" t="str">
-        <v>2 chiều</v>
+        <v>✓</v>
       </c>
       <c r="H40" t="str">
         <v>{{sla_C1_requirement}}</v>
@@ -1380,7 +1380,7 @@
         <v>R8c4</v>
       </c>
       <c r="G41" t="str">
-        <v>2 chiều</v>
+        <v>✓</v>
       </c>
       <c r="H41" t="str">
         <v>{{sla_C1_target}}</v>
@@ -1406,7 +1406,7 @@
         <v>R8c6</v>
       </c>
       <c r="G42" t="str">
-        <v>2 chiều (điền khi nghiệm thu)</v>
+        <v>Nghiệm thu</v>
       </c>
       <c r="H42" t="str">
         <v>{{sla_C1_score}}</v>
@@ -1432,7 +1432,7 @@
         <v>R8c7</v>
       </c>
       <c r="G43" t="str">
-        <v>2 chiều (điền khi nghiệm thu)</v>
+        <v>Nghiệm thu</v>
       </c>
       <c r="H43" t="str">
         <v>{{sla_C1_note}}</v>
@@ -1458,7 +1458,7 @@
         <v>R9c1</v>
       </c>
       <c r="G44" t="str">
-        <v>2 chiều</v>
+        <v>✓</v>
       </c>
       <c r="H44" t="str">
         <v>{{sla_C2_name}}</v>
@@ -1484,7 +1484,7 @@
         <v>R9c2</v>
       </c>
       <c r="G45" t="str">
-        <v>2 chiều</v>
+        <v>✓</v>
       </c>
       <c r="H45" t="str">
         <v>{{sla_C2_requirement}}</v>
@@ -1510,7 +1510,7 @@
         <v>R9c4</v>
       </c>
       <c r="G46" t="str">
-        <v>2 chiều</v>
+        <v>✓</v>
       </c>
       <c r="H46" t="str">
         <v>{{sla_C2_target}}</v>
@@ -1536,7 +1536,7 @@
         <v>R9c6</v>
       </c>
       <c r="G47" t="str">
-        <v>2 chiều (điền khi nghiệm thu)</v>
+        <v>Nghiệm thu</v>
       </c>
       <c r="H47" t="str">
         <v>{{sla_C2_score}}</v>
@@ -1562,7 +1562,7 @@
         <v>R9c7</v>
       </c>
       <c r="G48" t="str">
-        <v>2 chiều (điền khi nghiệm thu)</v>
+        <v>Nghiệm thu</v>
       </c>
       <c r="H48" t="str">
         <v>{{sla_C2_note}}</v>
@@ -1588,7 +1588,7 @@
         <v>R10c1</v>
       </c>
       <c r="G49" t="str">
-        <v>2 chiều</v>
+        <v>✓</v>
       </c>
       <c r="H49" t="str">
         <v>{{sla_C3_name}}</v>
@@ -1614,7 +1614,7 @@
         <v>R10c2</v>
       </c>
       <c r="G50" t="str">
-        <v>2 chiều</v>
+        <v>✓</v>
       </c>
       <c r="H50" t="str">
         <v>{{sla_C3_requirement}}</v>
@@ -1640,7 +1640,7 @@
         <v>R10c4</v>
       </c>
       <c r="G51" t="str">
-        <v>2 chiều</v>
+        <v>✓</v>
       </c>
       <c r="H51" t="str">
         <v>{{sla_C3_target}}</v>
@@ -1666,7 +1666,7 @@
         <v>R10c6</v>
       </c>
       <c r="G52" t="str">
-        <v>2 chiều (điền khi nghiệm thu)</v>
+        <v>Nghiệm thu</v>
       </c>
       <c r="H52" t="str">
         <v>{{sla_C3_score}}</v>
@@ -1692,7 +1692,7 @@
         <v>R10c7</v>
       </c>
       <c r="G53" t="str">
-        <v>2 chiều (điền khi nghiệm thu)</v>
+        <v>Nghiệm thu</v>
       </c>
       <c r="H53" t="str">
         <v>{{sla_C3_note}}</v>
@@ -1718,7 +1718,7 @@
         <v>R11c1</v>
       </c>
       <c r="G54" t="str">
-        <v>2 chiều</v>
+        <v>✓</v>
       </c>
       <c r="H54" t="str">
         <v>{{sla_C4_name}}</v>
@@ -1744,7 +1744,7 @@
         <v>R11c2</v>
       </c>
       <c r="G55" t="str">
-        <v>2 chiều</v>
+        <v>✓</v>
       </c>
       <c r="H55" t="str">
         <v>{{sla_C4_requirement}}</v>
@@ -1770,7 +1770,7 @@
         <v>R11c4</v>
       </c>
       <c r="G56" t="str">
-        <v>2 chiều</v>
+        <v>✓</v>
       </c>
       <c r="H56" t="str">
         <v>{{sla_C4_target}}</v>
@@ -1796,7 +1796,7 @@
         <v>R11c6</v>
       </c>
       <c r="G57" t="str">
-        <v>2 chiều (điền khi nghiệm thu)</v>
+        <v>Nghiệm thu</v>
       </c>
       <c r="H57" t="str">
         <v>{{sla_C4_score}}</v>
@@ -1822,7 +1822,7 @@
         <v>R11c7</v>
       </c>
       <c r="G58" t="str">
-        <v>2 chiều (điền khi nghiệm thu)</v>
+        <v>Nghiệm thu</v>
       </c>
       <c r="H58" t="str">
         <v>{{sla_C4_note}}</v>

</xml_diff>